<commit_message>
Mover modulo Tesoreria de Fase Starter (6 modulos) a Fase Express (14 modulos)
</commit_message>
<xml_diff>
--- a/Matriz_de_Evolucion_Operativa 2.xlsx
+++ b/Matriz_de_Evolucion_Operativa 2.xlsx
@@ -1382,8 +1382,16 @@
         </is>
       </c>
       <c r="B14" s="28" t="n"/>
-      <c r="C14" s="28" t="n"/>
-      <c r="D14" s="28" t="n"/>
+      <c r="C14" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D14" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="E14" s="28" t="inlineStr">
         <is>
           <t>X</t>

</xml_diff>

<commit_message>
Incluir modulo BI Cubo OLAP (BI y Reportes) en Fase 3 Advanced (19 modulos)
</commit_message>
<xml_diff>
--- a/Matriz_de_Evolucion_Operativa 2.xlsx
+++ b/Matriz_de_Evolucion_Operativa 2.xlsx
@@ -1418,7 +1418,11 @@
       </c>
       <c r="B16" s="28" t="n"/>
       <c r="C16" s="28" t="n"/>
-      <c r="D16" s="28" t="n"/>
+      <c r="D16" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="E16" s="28" t="inlineStr">
         <is>
           <t>X</t>

</xml_diff>